<commit_message>
atualização graficos e dados e ajustes finais
</commit_message>
<xml_diff>
--- a/dados/rgf_estados_2015_2025.xlsx
+++ b/dados/rgf_estados_2015_2025.xlsx
@@ -23278,9 +23278,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
         <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -27273,9 +27273,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
         <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
melhorias no notebook de analise.
</commit_message>
<xml_diff>
--- a/dados/rgf_estados_2015_2025.xlsx
+++ b/dados/rgf_estados_2015_2025.xlsx
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>3.849999999999994</v>
+        <v>3.849999999999993</v>
       </c>
       <c r="R3" t="n">
         <v>6.299999999999997</v>
@@ -925,7 +925,7 @@
         <v>49</v>
       </c>
       <c r="O6" t="n">
-        <v>43.41630648157631</v>
+        <v>43.41630648157632</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
         <v>49</v>
       </c>
       <c r="O11" t="n">
-        <v>46.23025961253948</v>
+        <v>46.23025961253949</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>-0.230000000000004</v>
+        <v>-0.2300000000000039</v>
       </c>
       <c r="R13" t="n">
         <v>2.219999999999999</v>
@@ -1729,7 +1729,7 @@
         <v>-1.270000000000003</v>
       </c>
       <c r="R17" t="n">
-        <v>1.18</v>
+        <v>1.179999999999999</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>-1.43</v>
+        <v>-1.429999999999999</v>
       </c>
       <c r="R19" t="n">
         <v>1.020000000000003</v>
@@ -2010,7 +2010,7 @@
         <v>49</v>
       </c>
       <c r="O21" t="n">
-        <v>48.34873470264075</v>
+        <v>48.34873470264076</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
         <v>48.6</v>
       </c>
       <c r="O22" t="n">
-        <v>48.43608150557723</v>
+        <v>48.43608150557724</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -2969,7 +2969,7 @@
         <v>49</v>
       </c>
       <c r="O34" t="n">
-        <v>42.67925134567012</v>
+        <v>42.67925134567013</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
         <v>5.670000000000002</v>
       </c>
       <c r="S36" t="n">
-        <v>-0.06000000000000227</v>
+        <v>-0.0600000000000022</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         <v>1.159999999999997</v>
       </c>
       <c r="R41" t="n">
-        <v>3.609999999999999</v>
+        <v>3.61</v>
       </c>
       <c r="S41" t="n">
         <v>-0.8399999999999963</v>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>-0.1499999999999986</v>
+        <v>-0.1499999999999985</v>
       </c>
       <c r="R44" t="n">
         <v>2.280000000000001</v>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>0.1499999999999986</v>
+        <v>0.1499999999999985</v>
       </c>
       <c r="R45" t="n">
         <v>2.600000000000001</v>
@@ -3880,7 +3880,7 @@
         <v>-0.5700000000000003</v>
       </c>
       <c r="R46" t="n">
-        <v>1.859999999999999</v>
+        <v>1.86</v>
       </c>
       <c r="S46" t="n">
         <v>-1.699999999999996</v>
@@ -3958,7 +3958,7 @@
         <v>2.18</v>
       </c>
       <c r="S47" t="n">
-        <v>0.03999999999999915</v>
+        <v>0.0399999999999991</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -4621,7 +4621,7 @@
         <v>48.6</v>
       </c>
       <c r="O56" t="n">
-        <v>39.30232299133691</v>
+        <v>39.30232299133692</v>
       </c>
       <c r="P56" t="inlineStr">
         <is>
@@ -5097,7 +5097,7 @@
         <v>5.700000000000003</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.03000000000000114</v>
+        <v>-0.0300000000000011</v>
       </c>
       <c r="T62" t="inlineStr">
         <is>
@@ -5328,7 +5328,7 @@
         <v>3.520000000000003</v>
       </c>
       <c r="S65" t="n">
-        <v>0.4600000000000009</v>
+        <v>0.4600000000000008</v>
       </c>
       <c r="T65" t="inlineStr">
         <is>
@@ -5458,7 +5458,7 @@
         <v>49</v>
       </c>
       <c r="O67" t="n">
-        <v>46.06909251884095</v>
+        <v>46.06909251884096</v>
       </c>
       <c r="P67" t="inlineStr">
         <is>
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>0.00999999999999801</v>
+        <v>0.009999999999998</v>
       </c>
       <c r="R68" t="n">
         <v>2.460000000000001</v>
@@ -6085,7 +6085,7 @@
         <v>-2.420000000000002</v>
       </c>
       <c r="R75" t="n">
-        <v>0.03000000000000114</v>
+        <v>0.0300000000000011</v>
       </c>
       <c r="S75" t="n">
         <v>3.199999999999996</v>
@@ -6162,7 +6162,7 @@
         <v>-2.440000000000005</v>
       </c>
       <c r="R76" t="n">
-        <v>0.00999999999999801</v>
+        <v>0.009999999999998</v>
       </c>
       <c r="S76" t="n">
         <v>5.840000000000003</v>
@@ -6239,7 +6239,7 @@
         <v>-2.440000000000005</v>
       </c>
       <c r="R77" t="n">
-        <v>0.00999999999999801</v>
+        <v>0.009999999999998</v>
       </c>
       <c r="S77" t="n">
         <v>6.310000000000002</v>
@@ -6316,7 +6316,7 @@
         <v>-3.420000000000002</v>
       </c>
       <c r="R78" t="n">
-        <v>-0.9699999999999989</v>
+        <v>-0.9699999999999988</v>
       </c>
       <c r="S78" t="n">
         <v>2.159999999999997</v>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>4.629999999999995</v>
+        <v>4.629999999999996</v>
       </c>
       <c r="R86" t="n">
         <v>7.079999999999998</v>
@@ -7012,7 +7012,7 @@
         <v>6.700000000000003</v>
       </c>
       <c r="S87" t="n">
-        <v>-0.1500000000000057</v>
+        <v>-0.1500000000000056</v>
       </c>
       <c r="T87" t="inlineStr">
         <is>
@@ -7089,7 +7089,7 @@
         <v>5.640000000000001</v>
       </c>
       <c r="S88" t="n">
-        <v>-0.07000000000000028</v>
+        <v>-0.0700000000000002</v>
       </c>
       <c r="T88" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
         </is>
       </c>
       <c r="Q93" t="n">
-        <v>0.03999999999999915</v>
+        <v>0.0399999999999991</v>
       </c>
       <c r="R93" t="n">
         <v>2.469999999999999</v>
@@ -7545,13 +7545,13 @@
         </is>
       </c>
       <c r="Q94" t="n">
-        <v>-0.04000000000000625</v>
+        <v>-0.0400000000000062</v>
       </c>
       <c r="R94" t="n">
         <v>2.409999999999997</v>
       </c>
       <c r="S94" t="n">
-        <v>0.05000000000000426</v>
+        <v>0.0500000000000042</v>
       </c>
       <c r="T94" t="inlineStr">
         <is>
@@ -7699,7 +7699,7 @@
         </is>
       </c>
       <c r="Q96" t="n">
-        <v>-0.9899999999999949</v>
+        <v>-0.9899999999999948</v>
       </c>
       <c r="R96" t="n">
         <v>1.440000000000005</v>
@@ -7845,7 +7845,7 @@
         <v>49</v>
       </c>
       <c r="O98" t="n">
-        <v>47.52285145517516</v>
+        <v>47.52285145517517</v>
       </c>
       <c r="P98" t="inlineStr">
         <is>
@@ -7859,7 +7859,7 @@
         <v>1.479999999999997</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.1299999999999955</v>
+        <v>-0.1299999999999954</v>
       </c>
       <c r="T98" t="inlineStr">
         <is>
@@ -8244,7 +8244,7 @@
         <v>0.3100000000000023</v>
       </c>
       <c r="S103" t="n">
-        <v>0.05999999999999517</v>
+        <v>0.0599999999999951</v>
       </c>
       <c r="T103" t="inlineStr">
         <is>
@@ -9011,7 +9011,7 @@
         <v>6.68</v>
       </c>
       <c r="R113" t="n">
-        <v>9.130000000000003</v>
+        <v>9.130000000000004</v>
       </c>
       <c r="S113" t="n">
         <v>-2.050000000000004</v>
@@ -9701,7 +9701,7 @@
         </is>
       </c>
       <c r="Q122" t="n">
-        <v>0.9499999999999957</v>
+        <v>0.9499999999999956</v>
       </c>
       <c r="R122" t="n">
         <v>3.399999999999999</v>
@@ -9932,7 +9932,7 @@
         </is>
       </c>
       <c r="Q125" t="n">
-        <v>-0.2900000000000063</v>
+        <v>-0.2900000000000062</v>
       </c>
       <c r="R125" t="n">
         <v>2.159999999999997</v>
@@ -10169,7 +10169,7 @@
         <v>1.920000000000002</v>
       </c>
       <c r="S128" t="n">
-        <v>-0.1400000000000006</v>
+        <v>-0.1400000000000005</v>
       </c>
       <c r="T128" t="inlineStr">
         <is>
@@ -10240,7 +10240,7 @@
         </is>
       </c>
       <c r="Q129" t="n">
-        <v>-1.57</v>
+        <v>-1.570000000000001</v>
       </c>
       <c r="R129" t="n">
         <v>0.8800000000000026</v>
@@ -10320,7 +10320,7 @@
         <v>-2.310000000000002</v>
       </c>
       <c r="R130" t="n">
-        <v>0.1400000000000006</v>
+        <v>0.1400000000000005</v>
       </c>
       <c r="S130" t="n">
         <v>-1.75</v>
@@ -10477,7 +10477,7 @@
         <v>-0.6499999999999986</v>
       </c>
       <c r="S132" t="n">
-        <v>1.32</v>
+        <v>1.320000000000001</v>
       </c>
       <c r="T132" t="inlineStr">
         <is>
@@ -10694,7 +10694,7 @@
         <v>49</v>
       </c>
       <c r="O135" t="n">
-        <v>58.41845547721667</v>
+        <v>58.41845547721668</v>
       </c>
       <c r="P135" t="inlineStr">
         <is>
@@ -10779,7 +10779,7 @@
         </is>
       </c>
       <c r="Q136" t="n">
-        <v>-14.01000000000001</v>
+        <v>-14.01</v>
       </c>
       <c r="R136" t="n">
         <v>-11.56</v>
@@ -11244,7 +11244,7 @@
         <v>6.769999999999996</v>
       </c>
       <c r="R142" t="n">
-        <v>9.219999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="S142" t="n">
         <v>-4.93</v>
@@ -11541,7 +11541,7 @@
         <v>49</v>
       </c>
       <c r="O146" t="n">
-        <v>42.05437635288268</v>
+        <v>42.05437635288269</v>
       </c>
       <c r="P146" t="inlineStr">
         <is>
@@ -11934,7 +11934,7 @@
         </is>
       </c>
       <c r="Q151" t="n">
-        <v>1.629999999999995</v>
+        <v>1.629999999999996</v>
       </c>
       <c r="R151" t="n">
         <v>4.079999999999998</v>
@@ -12165,7 +12165,7 @@
         </is>
       </c>
       <c r="Q154" t="n">
-        <v>1.07</v>
+        <v>1.070000000000001</v>
       </c>
       <c r="R154" t="n">
         <v>3.520000000000003</v>
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="Q157" t="n">
-        <v>0.01999999999999602</v>
+        <v>0.019999999999996</v>
       </c>
       <c r="R157" t="n">
         <v>2.469999999999999</v>
@@ -12850,7 +12850,7 @@
         <v>49</v>
       </c>
       <c r="O163" t="n">
-        <v>54.81200404936511</v>
+        <v>54.81200404936512</v>
       </c>
       <c r="P163" t="inlineStr">
         <is>
@@ -12935,7 +12935,7 @@
         </is>
       </c>
       <c r="Q164" t="n">
-        <v>11.73999999999999</v>
+        <v>11.74</v>
       </c>
       <c r="R164" t="n">
         <v>14.19</v>
@@ -13249,7 +13249,7 @@
         <v>11.54</v>
       </c>
       <c r="S168" t="n">
-        <v>-0.04999999999999716</v>
+        <v>-0.0499999999999971</v>
       </c>
       <c r="T168" t="inlineStr">
         <is>
@@ -13403,7 +13403,7 @@
         <v>10.32</v>
       </c>
       <c r="S170" t="n">
-        <v>-6.629999999999995</v>
+        <v>-6.629999999999996</v>
       </c>
       <c r="T170" t="inlineStr">
         <is>
@@ -14236,7 +14236,7 @@
         <v>49</v>
       </c>
       <c r="O181" t="n">
-        <v>41.3693139045814</v>
+        <v>41.36931390458141</v>
       </c>
       <c r="P181" t="inlineStr">
         <is>
@@ -14250,7 +14250,7 @@
         <v>7.630000000000003</v>
       </c>
       <c r="S181" t="n">
-        <v>-1.120000000000005</v>
+        <v>-1.120000000000004</v>
       </c>
       <c r="T181" t="inlineStr">
         <is>
@@ -14629,7 +14629,7 @@
         </is>
       </c>
       <c r="Q186" t="n">
-        <v>-0.1500000000000057</v>
+        <v>-0.1500000000000056</v>
       </c>
       <c r="R186" t="n">
         <v>2.299999999999997</v>
@@ -15091,7 +15091,7 @@
         </is>
       </c>
       <c r="Q192" t="n">
-        <v>9.969999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="R192" t="n">
         <v>12.4</v>
@@ -15479,7 +15479,7 @@
         <v>7.419999999999995</v>
       </c>
       <c r="R197" t="n">
-        <v>9.869999999999997</v>
+        <v>9.869999999999996</v>
       </c>
       <c r="S197" t="n">
         <v>-1.489999999999995</v>
@@ -15633,7 +15633,7 @@
         <v>7.199999999999996</v>
       </c>
       <c r="R199" t="n">
-        <v>9.649999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="S199" t="n">
         <v>-0.9600000000000009</v>
@@ -16315,7 +16315,7 @@
         <v>49</v>
       </c>
       <c r="O208" t="n">
-        <v>43.03264508562292</v>
+        <v>43.03264508562293</v>
       </c>
       <c r="P208" t="inlineStr">
         <is>
@@ -16777,7 +16777,7 @@
         <v>49</v>
       </c>
       <c r="O214" t="n">
-        <v>46.35909143224244</v>
+        <v>46.35909143224245</v>
       </c>
       <c r="P214" t="inlineStr">
         <is>
@@ -17247,7 +17247,7 @@
         </is>
       </c>
       <c r="Q220" t="n">
-        <v>9.049999999999997</v>
+        <v>9.049999999999995</v>
       </c>
       <c r="R220" t="n">
         <v>11.5</v>
@@ -17632,13 +17632,13 @@
         </is>
       </c>
       <c r="Q225" t="n">
-        <v>6.379999999999995</v>
+        <v>6.379999999999996</v>
       </c>
       <c r="R225" t="n">
         <v>8.829999999999998</v>
       </c>
       <c r="S225" t="n">
-        <v>-0.9299999999999997</v>
+        <v>-0.9299999999999996</v>
       </c>
       <c r="T225" t="inlineStr">
         <is>
@@ -18479,13 +18479,13 @@
         </is>
       </c>
       <c r="Q236" t="n">
-        <v>1.82</v>
+        <v>1.820000000000001</v>
       </c>
       <c r="R236" t="n">
         <v>4.270000000000003</v>
       </c>
       <c r="S236" t="n">
-        <v>1.899999999999999</v>
+        <v>1.899999999999998</v>
       </c>
       <c r="T236" t="inlineStr">
         <is>
@@ -18556,7 +18556,7 @@
         </is>
       </c>
       <c r="Q237" t="n">
-        <v>1.68</v>
+        <v>1.679999999999999</v>
       </c>
       <c r="R237" t="n">
         <v>4.130000000000003</v>
@@ -18710,7 +18710,7 @@
         </is>
       </c>
       <c r="Q239" t="n">
-        <v>-0.9200000000000017</v>
+        <v>-0.9200000000000016</v>
       </c>
       <c r="R239" t="n">
         <v>1.530000000000001</v>
@@ -18864,7 +18864,7 @@
         </is>
       </c>
       <c r="Q241" t="n">
-        <v>-1.859999999999999</v>
+        <v>-1.86</v>
       </c>
       <c r="R241" t="n">
         <v>0.5900000000000034</v>
@@ -20256,7 +20256,7 @@
         <v>6.810000000000002</v>
       </c>
       <c r="S259" t="n">
-        <v>-0.1400000000000006</v>
+        <v>-0.1400000000000005</v>
       </c>
       <c r="T259" t="inlineStr">
         <is>
@@ -20712,7 +20712,7 @@
         </is>
       </c>
       <c r="Q265" t="n">
-        <v>0.2299999999999969</v>
+        <v>0.2299999999999968</v>
       </c>
       <c r="R265" t="n">
         <v>2.68</v>
@@ -20789,7 +20789,7 @@
         </is>
       </c>
       <c r="Q266" t="n">
-        <v>-0.2100000000000009</v>
+        <v>-0.2100000000000008</v>
       </c>
       <c r="R266" t="n">
         <v>2.240000000000002</v>
@@ -20866,13 +20866,13 @@
         </is>
       </c>
       <c r="Q267" t="n">
-        <v>-0.220000000000006</v>
+        <v>-0.2200000000000059</v>
       </c>
       <c r="R267" t="n">
         <v>2.229999999999997</v>
       </c>
       <c r="S267" t="n">
-        <v>-1.639999999999993</v>
+        <v>-1.639999999999994</v>
       </c>
       <c r="T267" t="inlineStr">
         <is>
@@ -20935,7 +20935,7 @@
         <v>49</v>
       </c>
       <c r="O268" t="n">
-        <v>47.27491234109119</v>
+        <v>47.2749123410912</v>
       </c>
       <c r="P268" t="inlineStr">
         <is>
@@ -21026,7 +21026,7 @@
         <v>0.7299999999999969</v>
       </c>
       <c r="S269" t="n">
-        <v>0.3900000000000006</v>
+        <v>0.3900000000000005</v>
       </c>
       <c r="T269" t="inlineStr">
         <is>
@@ -21174,7 +21174,7 @@
         </is>
       </c>
       <c r="Q271" t="n">
-        <v>-11.01000000000001</v>
+        <v>-11.01</v>
       </c>
       <c r="R271" t="n">
         <v>-8.560000000000002</v>
@@ -21488,7 +21488,7 @@
         <v>11.2</v>
       </c>
       <c r="S275" t="n">
-        <v>-3.859999999999999</v>
+        <v>-3.86</v>
       </c>
       <c r="T275" t="inlineStr">
         <is>
@@ -21873,7 +21873,7 @@
         <v>10.28</v>
       </c>
       <c r="S280" t="n">
-        <v>-0.9399999999999977</v>
+        <v>-0.9399999999999976</v>
       </c>
       <c r="T280" t="inlineStr">
         <is>
@@ -22175,7 +22175,7 @@
         </is>
       </c>
       <c r="Q284" t="n">
-        <v>5.629999999999995</v>
+        <v>5.629999999999996</v>
       </c>
       <c r="R284" t="n">
         <v>8.079999999999998</v>
@@ -24044,7 +24044,7 @@
         <v>3.762727272727275</v>
       </c>
       <c r="P7" t="n">
-        <v>6.192727272727276</v>
+        <v>6.192727272727274</v>
       </c>
       <c r="Q7" t="n">
         <v>4</v>
@@ -28039,7 +28039,7 @@
         <v>3.762727272727275</v>
       </c>
       <c r="P7" t="n">
-        <v>6.192727272727276</v>
+        <v>6.192727272727274</v>
       </c>
       <c r="Q7" t="n">
         <v>4</v>
@@ -33670,7 +33670,7 @@
         <v>3.762727272727275</v>
       </c>
       <c r="P19" t="n">
-        <v>6.192727272727276</v>
+        <v>6.192727272727274</v>
       </c>
       <c r="Q19" t="n">
         <v>4</v>

</xml_diff>